<commit_message>
docs: finalize tracker split — dedup Epic 3 + persist Stability marks
The Stability tracker file was Excel-locked in the previous batch,
so the mark-items + SUPERSEDED-banner writes were deferred. Founder
closed the file; re-ran the restructure script:

- 5 Stability items now marked "Moved to Epic 3" in-place with
  pointers in Notes: S4-05, S4-06, S4-08, S4-09, FUP-47.
- Stability tracker README gets an ==> SUPERSEDED 2026-08-15 <==
  banner directing readers to the new per-epic files.

The re-run non-idempotently appended the 5 items to Epic 3 again
(18 rows instead of 13). Removed the duplicates via delete_rows +
restored Dashboard totals. Epic 3 now correctly shows 13 items
across 4 sprints. Master tracker Epic 3 row restored to 13.

All-epics rollup: 139/191 (73%).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic3_Dex_AI_Persona.xlsx
+++ b/docs/DecisionOS_Epic3_Dex_AI_Persona.xlsx
@@ -833,7 +833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1093,6 +1093,49 @@
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Sprint 4 -- Dex knowledge + retrieval (5 items imported from Epic 1 Stability tracker on 2026-08-15). Ingest-time document extraction + chunk + embed, vector search + hybrid retrieval, bounded planner-executor loop with native function-calling, per-conversation agent memory, auto-assign AI-generated tasks. Sits alongside the persona work in Sprint 1-3 -- this sprint is the 'how does Dex actually know things' layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>Sprint 4 -- Dex knowledge + retrieval</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Backlog (imported from Stability tracker 2026-08-15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>E3-09, E3-10, E3-11, E3-12, E3-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="100" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>Sprint 4 -- Dex knowledge + retrieval (5 items imported from Epic 1 Stability tracker on 2026-08-15). Ingest-time document extraction + chunk + embed, vector search + hybrid retrieval, bounded planner-executor loop with native function-calling, per-conversation agent memory, auto-assign AI-generated tasks. Sits alongside the persona work in Sprint 1-3 -- this sprint is the 'how does Dex actually know things' layer.</t>
         </is>
@@ -1907,6 +1950,11 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="180" customHeight="1"/>
+    <row r="16" ht="180" customHeight="1"/>
+    <row r="17" ht="180" customHeight="1"/>
+    <row r="18" ht="180" customHeight="1"/>
+    <row r="19" ht="180" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>